<commit_message>
Update manual excel with interactive dropdown selection
</commit_message>
<xml_diff>
--- a/ENCUESTA_MANUAL_PYME.xlsx
+++ b/ENCUESTA_MANUAL_PYME.xlsx
@@ -645,7 +645,7 @@
       <c r="C13" s="8" t="n"/>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Sí, ingresé y participé de las presentaciones y conversatorios. | Sí, pero no participé de nada adicional. | No, entré por otra vía.</t>
+          <t>Sí - ingresé y participé de las presentaciones y conversatorios. | Sí - pero no participé de nada adicional. | No - entré por otra vía.</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>No, desconozco qué es el Fill Rate | Sí, sé qué es, pero no lo sigo | Sí, lo conozco y reviso ocasionalmente | Sí, lo reviso y gestiono activamente</t>
+          <t>No - desconozco qué es el Fill Rate | Sí - sé qué es - pero no lo sigo | Sí - lo conozco y reviso ocasionalmente | Sí - lo reviso y gestiono activamente</t>
         </is>
       </c>
     </row>
@@ -677,7 +677,7 @@
       <c r="C15" s="8" t="n"/>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>No, no lo conozco | Sí, lo conozco pero no lo monitoreo activamente | Sí, lo monitoreo activamente</t>
+          <t>No - no lo conozco | Sí - lo conozco pero no lo monitoreo activamente | Sí - lo monitoreo activamente</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       <c r="C16" s="8" t="n"/>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>No, no conozco bien los requisitos de entrega | Conozco algunos pero tengo dudas frecuentes | Sí, los conozco y los cumplo correctamente</t>
+          <t>No - no conozco bien los requisitos de entrega | Conozco algunos pero tengo dudas frecuentes | Sí - los conozco y los cumplo correctamente</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       <c r="C17" s="8" t="n"/>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>No, desconozco el proceso de agendamiento | Sí, pero tengo dudas frecuentes | Sí, lo sé y lo hago sin problemas</t>
+          <t>No - desconozco el proceso de agendamiento | Sí - pero tengo dudas frecuentes | Sí - lo sé y lo hago sin problemas</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       <c r="C18" s="8" t="n"/>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>No, no tengo esa información | Sí, pero solo cuando me avisan del quiebre | Sí, lo monitoreo regularmente</t>
+          <t>No - no tengo esa información | Sí - pero solo cuando me avisan del quiebre | Sí - lo monitoreo regularmente</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       <c r="C19" s="8" t="n"/>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>No tengo visibilidad de mis quiebres | Sí, frecuentemente (más de 1 vez/mes) | Sí, ocurren ocasionalmente | Sí, ocurren rara vez</t>
+          <t>No tengo visibilidad de mis quiebres | Sí - frecuentemente (más de 1 vez/mes) | Sí - ocurren ocasionalmente | Sí - ocurren rara vez</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       <c r="C20" s="8" t="n"/>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>No, no tengo acceso | Sí, tengo acceso pero no sé para qué me sirve | Sí, lo uso para cosas básicas | Sí, lo uso y aprovecho sus reportes</t>
+          <t>No - no tengo acceso | Sí - tengo acceso pero no sé para qué me sirve | Sí - lo uso para cosas básicas | Sí - lo uso y aprovecho sus reportes</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       <c r="C22" s="8" t="n"/>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>No, nunca he escuchado ese nombre | Sí, lo conozco pero no lo uso | Sí, lo uso y sé cómo funciona</t>
+          <t>No - nunca he escuchado ese nombre | Sí - lo conozco pero no lo uso | Sí - lo uso y sé cómo funciona</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>No, no sé en qué tiendas estoy | Sé en cuáles tiendas estoy pero no lo actualizo | Sí, tengo información actualizada de mi presencia | Sí, además monitoreo el desempeño por local</t>
+          <t>No - no sé en qué tiendas estoy | Sé en cuáles tiendas estoy pero no lo actualizo | Sí - tengo información actualizada de mi presencia | Sí - además monitoreo el desempeño por local</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>No, no conozco el proceso | He escuchado del proceso pero no lo conozco en detalle | Sí, lo conozco pero aún no he realizado alzas | Sí, he realizado alzas y conozco bien el proceso</t>
+          <t>No - no conozco el proceso | He escuchado del proceso pero no lo conozco en detalle | Sí - lo conozco pero aún no he realizado alzas | Sí - he realizado alzas y conozco bien el proceso</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>No, nunca he participado | No, desconozco los requisitos | Sí, pero solo cuando me invitan | Sí, las busco activamente</t>
+          <t>No - nunca he participado | No - desconozco los requisitos | Sí - pero solo cuando me invitan | Sí - las busco activamente</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
       <c r="C26" s="8" t="n"/>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>No, no entiendo la diferencia | Tengo una idea general pero no claridad total | Sí, los diferencio claramente</t>
+          <t>No - no entiendo la diferencia | Tengo una idea general pero no claridad total | Sí - los diferencio claramente</t>
         </is>
       </c>
     </row>
@@ -885,7 +885,7 @@
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>No, no lo conozco | Sí, he escuchado de él pero no sé cómo funciona | Sí, lo conozco y me interesa participar | Sí, ya participo o he participado en él</t>
+          <t>No - no lo conozco | Sí - he escuchado de él pero no sé cómo funciona | Sí - lo conozco y me interesa participar | Sí - ya participo o he participado en él</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>No, no sé a quién acudir | Sí, tengo un contacto principal | Sí, tengo contactos según el tema</t>
+          <t>No - no sé a quién acudir | Sí - tengo un contacto principal | Sí - tengo contactos según el tema</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>No, rara vez obtengo respuesta | Sí, a veces depende del tema | Sí, siempre obtengo respuesta oportuna</t>
+          <t>No - rara vez obtengo respuesta | Sí - a veces depende del tema | Sí - siempre obtengo respuesta oportuna</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>No, no entiendo los motivos del rechazo | Sí, entiendo pero me cuesta corregirlo | Sí, entiendo y corrijo de inmediato</t>
+          <t>No - no entiendo los motivos del rechazo | Sí - entiendo pero me cuesta corregirlo | Sí - entiendo y corrijo de inmediato</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       <c r="C32" s="8" t="n"/>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>No, no sé qué es | Sí, lo conozco pero no entiendo bien por qué | Sí, lo conozco y entiendo por qué se cobra</t>
+          <t>No - no sé qué es | Sí - lo conozco pero no entiendo bien por qué | Sí - lo conozco y entiendo por qué se cobra</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>No, no sé qué es | Sí, lo conozco pero no entiendo bien por qué | Sí, lo conozco y entiendo por qué se cobra</t>
+          <t>No - no sé qué es | Sí - lo conozco pero no entiendo bien por qué | Sí - lo conozco y entiendo por qué se cobra</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Sí, contamos con certificación | No, no tenemos certificación | En proceso de certificación</t>
+          <t>Sí - contamos con certificación | No - no tenemos certificación | En proceso de certificación</t>
         </is>
       </c>
     </row>
@@ -990,6 +990,80 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D3"/>
   </mergeCells>
+  <dataValidations count="24">
+    <dataValidation sqref="C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"Alimentos y Bebidas,Limpieza y Hogar,Cuidado Personal,Textil y Ropa,Electrónica,Otra categoría"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"Menos de 6 meses,Entre 6 meses y 1 año,Entre 1 y 3 años,Más de 3 años"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"Sí - ingresé y participé de las presentaciones y conversatorios.,Sí - pero no participé de nada adicional.,No - entré por otra vía."</formula1>
+    </dataValidation>
+    <dataValidation sqref="C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - desconozco qué es el Fill Rate,Sí - sé qué es - pero no lo sigo,Sí - lo conozco y reviso ocasionalmente,Sí - lo reviso y gestiono activamente"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no lo conozco,Sí - lo conozco pero no lo monitoreo activamente,Sí - lo monitoreo activamente"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no conozco bien los requisitos de entrega,Conozco algunos pero tengo dudas frecuentes,Sí - los conozco y los cumplo correctamente"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - desconozco el proceso de agendamiento,Sí - pero tengo dudas frecuentes,Sí - lo sé y lo hago sin problemas"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no tengo esa información,Sí - pero solo cuando me avisan del quiebre,Sí - lo monitoreo regularmente"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No tengo visibilidad de mis quiebres,Sí - frecuentemente (más de 1 vez/mes),Sí - ocurren ocasionalmente,Sí - ocurren rara vez"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no tengo acceso,Sí - tengo acceso pero no sé para qué me sirve,Sí - lo uso para cosas básicas,Sí - lo uso y aprovecho sus reportes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No lo hago,Una vez al mes,Semanalmente,Diariamente"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - nunca he escuchado ese nombre,Sí - lo conozco pero no lo uso,Sí - lo uso y sé cómo funciona"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no sé en qué tiendas estoy,Sé en cuáles tiendas estoy pero no lo actualizo,Sí - tengo información actualizada de mi presencia,Sí - además monitoreo el desempeño por local"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no conozco el proceso,He escuchado del proceso pero no lo conozco en detalle,Sí - lo conozco pero aún no he realizado alzas,Sí - he realizado alzas y conozco bien el proceso"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - nunca he participado,No - desconozco los requisitos,Sí - pero solo cuando me invitan,Sí - las busco activamente"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no entiendo la diferencia,Tengo una idea general pero no claridad total,Sí - los diferencio claramente"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"Soy yo quien administra la cuenta,Tengo KAM especializado para la cuenta,Tengo un conocido para la cuenta"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no lo conozco,Sí - he escuchado de él pero no sé cómo funciona,Sí - lo conozco y me interesa participar,Sí - ya participo o he participado en él"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no sé a quién acudir,Sí - tengo un contacto principal,Sí - tengo contactos según el tema"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - rara vez obtengo respuesta,Sí - a veces depende del tema,Sí - siempre obtengo respuesta oportuna"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no entiendo los motivos del rechazo,Sí - entiendo pero me cuesta corregirlo,Sí - entiendo y corrijo de inmediato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no sé qué es,Sí - lo conozco pero no entiendo bien por qué,Sí - lo conozco y entiendo por qué se cobra"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"No - no sé qué es,Sí - lo conozco pero no entiendo bien por qué,Sí - lo conozco y entiendo por qué se cobra"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
+      <formula1>"Sí - contamos con certificación,No - no tenemos certificación,En proceso de certificación"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix excel manual dropdown validation with hidden reference sheet
</commit_message>
<xml_diff>
--- a/ENCUESTA_MANUAL_PYME.xlsx
+++ b/ENCUESTA_MANUAL_PYME.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Encuesta PyME Offline" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opciones_Encuesta" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -645,7 +646,7 @@
       <c r="C13" s="8" t="n"/>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Sí - ingresé y participé de las presentaciones y conversatorios. | Sí - pero no participé de nada adicional. | No - entré por otra vía.</t>
+          <t>Sí, ingresé y participé de las presentaciones y conversatorios. | Sí, pero no participé de nada adicional. | No, entré por otra vía.</t>
         </is>
       </c>
     </row>
@@ -661,7 +662,7 @@
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>No - desconozco qué es el Fill Rate | Sí - sé qué es - pero no lo sigo | Sí - lo conozco y reviso ocasionalmente | Sí - lo reviso y gestiono activamente</t>
+          <t>No, desconozco qué es el Fill Rate | Sí, sé qué es, pero no lo sigo | Sí, lo conozco y reviso ocasionalmente | Sí, lo reviso y gestiono activamente</t>
         </is>
       </c>
     </row>
@@ -677,7 +678,7 @@
       <c r="C15" s="8" t="n"/>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>No - no lo conozco | Sí - lo conozco pero no lo monitoreo activamente | Sí - lo monitoreo activamente</t>
+          <t>No, no lo conozco | Sí, lo conozco pero no lo monitoreo activamente | Sí, lo monitoreo activamente</t>
         </is>
       </c>
     </row>
@@ -693,7 +694,7 @@
       <c r="C16" s="8" t="n"/>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>No - no conozco bien los requisitos de entrega | Conozco algunos pero tengo dudas frecuentes | Sí - los conozco y los cumplo correctamente</t>
+          <t>No, no conozco bien los requisitos de entrega | Conozco algunos pero tengo dudas frecuentes | Sí, los conozco y los cumplo correctamente</t>
         </is>
       </c>
     </row>
@@ -709,7 +710,7 @@
       <c r="C17" s="8" t="n"/>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>No - desconozco el proceso de agendamiento | Sí - pero tengo dudas frecuentes | Sí - lo sé y lo hago sin problemas</t>
+          <t>No, desconozco el proceso de agendamiento | Sí, pero tengo dudas frecuentes | Sí, lo sé y lo hago sin problemas</t>
         </is>
       </c>
     </row>
@@ -725,7 +726,7 @@
       <c r="C18" s="8" t="n"/>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>No - no tengo esa información | Sí - pero solo cuando me avisan del quiebre | Sí - lo monitoreo regularmente</t>
+          <t>No, no tengo esa información | Sí, pero solo cuando me avisan del quiebre | Sí, lo monitoreo regularmente</t>
         </is>
       </c>
     </row>
@@ -741,7 +742,7 @@
       <c r="C19" s="8" t="n"/>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>No tengo visibilidad de mis quiebres | Sí - frecuentemente (más de 1 vez/mes) | Sí - ocurren ocasionalmente | Sí - ocurren rara vez</t>
+          <t>No tengo visibilidad de mis quiebres | Sí, frecuentemente (más de 1 vez/mes) | Sí, ocurren ocasionalmente | Sí, ocurren rara vez</t>
         </is>
       </c>
     </row>
@@ -757,7 +758,7 @@
       <c r="C20" s="8" t="n"/>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>No - no tengo acceso | Sí - tengo acceso pero no sé para qué me sirve | Sí - lo uso para cosas básicas | Sí - lo uso y aprovecho sus reportes</t>
+          <t>No, no tengo acceso | Sí, tengo acceso pero no sé para qué me sirve | Sí, lo uso para cosas básicas | Sí, lo uso y aprovecho sus reportes</t>
         </is>
       </c>
     </row>
@@ -789,7 +790,7 @@
       <c r="C22" s="8" t="n"/>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>No - nunca he escuchado ese nombre | Sí - lo conozco pero no lo uso | Sí - lo uso y sé cómo funciona</t>
+          <t>No, nunca he escuchado ese nombre | Sí, lo conozco pero no lo uso | Sí, lo uso y sé cómo funciona</t>
         </is>
       </c>
     </row>
@@ -805,7 +806,7 @@
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>No - no sé en qué tiendas estoy | Sé en cuáles tiendas estoy pero no lo actualizo | Sí - tengo información actualizada de mi presencia | Sí - además monitoreo el desempeño por local</t>
+          <t>No, no sé en qué tiendas estoy | Sé en cuáles tiendas estoy pero no lo actualizo | Sí, tengo información actualizada de mi presencia | Sí, además monitoreo el desempeño por local</t>
         </is>
       </c>
     </row>
@@ -821,7 +822,7 @@
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>No - no conozco el proceso | He escuchado del proceso pero no lo conozco en detalle | Sí - lo conozco pero aún no he realizado alzas | Sí - he realizado alzas y conozco bien el proceso</t>
+          <t>No, no conozco el proceso | He escuchado del proceso pero no lo conozco en detalle | Sí, lo conozco pero aún no he realizado alzas | Sí, he realizado alzas y conozco bien el proceso</t>
         </is>
       </c>
     </row>
@@ -837,7 +838,7 @@
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>No - nunca he participado | No - desconozco los requisitos | Sí - pero solo cuando me invitan | Sí - las busco activamente</t>
+          <t>No, nunca he participado | No, desconozco los requisitos | Sí, pero solo cuando me invitan | Sí, las busco activamente</t>
         </is>
       </c>
     </row>
@@ -853,7 +854,7 @@
       <c r="C26" s="8" t="n"/>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>No - no entiendo la diferencia | Tengo una idea general pero no claridad total | Sí - los diferencio claramente</t>
+          <t>No, no entiendo la diferencia | Tengo una idea general pero no claridad total | Sí, los diferencio claramente</t>
         </is>
       </c>
     </row>
@@ -885,7 +886,7 @@
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>No - no lo conozco | Sí - he escuchado de él pero no sé cómo funciona | Sí - lo conozco y me interesa participar | Sí - ya participo o he participado en él</t>
+          <t>No, no lo conozco | Sí, he escuchado de él pero no sé cómo funciona | Sí, lo conozco y me interesa participar | Sí, ya participo o he participado en él</t>
         </is>
       </c>
     </row>
@@ -901,7 +902,7 @@
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>No - no sé a quién acudir | Sí - tengo un contacto principal | Sí - tengo contactos según el tema</t>
+          <t>No, no sé a quién acudir | Sí, tengo un contacto principal | Sí, tengo contactos según el tema</t>
         </is>
       </c>
     </row>
@@ -917,7 +918,7 @@
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>No - rara vez obtengo respuesta | Sí - a veces depende del tema | Sí - siempre obtengo respuesta oportuna</t>
+          <t>No, rara vez obtengo respuesta | Sí, a veces depende del tema | Sí, siempre obtengo respuesta oportuna</t>
         </is>
       </c>
     </row>
@@ -933,7 +934,7 @@
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>No - no entiendo los motivos del rechazo | Sí - entiendo pero me cuesta corregirlo | Sí - entiendo y corrijo de inmediato</t>
+          <t>No, no entiendo los motivos del rechazo | Sí, entiendo pero me cuesta corregirlo | Sí, entiendo y corrijo de inmediato</t>
         </is>
       </c>
     </row>
@@ -949,7 +950,7 @@
       <c r="C32" s="8" t="n"/>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>No - no sé qué es | Sí - lo conozco pero no entiendo bien por qué | Sí - lo conozco y entiendo por qué se cobra</t>
+          <t>No, no sé qué es | Sí, lo conozco pero no entiendo bien por qué | Sí, lo conozco y entiendo por qué se cobra</t>
         </is>
       </c>
     </row>
@@ -965,7 +966,7 @@
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>No - no sé qué es | Sí - lo conozco pero no entiendo bien por qué | Sí - lo conozco y entiendo por qué se cobra</t>
+          <t>No, no sé qué es | Sí, lo conozco pero no entiendo bien por qué | Sí, lo conozco y entiendo por qué se cobra</t>
         </is>
       </c>
     </row>
@@ -981,7 +982,7 @@
       <c r="C34" s="8" t="n"/>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Sí - contamos con certificación | No - no tenemos certificación | En proceso de certificación</t>
+          <t>Sí, contamos con certificación | No, no tenemos certificación | En proceso de certificación</t>
         </is>
       </c>
     </row>
@@ -991,79 +992,525 @@
     <mergeCell ref="A2:D3"/>
   </mergeCells>
   <dataValidations count="24">
-    <dataValidation sqref="C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"Alimentos y Bebidas,Limpieza y Hogar,Cuidado Personal,Textil y Ropa,Electrónica,Otra categoría"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"Menos de 6 meses,Entre 6 meses y 1 año,Entre 1 y 3 años,Más de 3 años"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"Sí - ingresé y participé de las presentaciones y conversatorios.,Sí - pero no participé de nada adicional.,No - entré por otra vía."</formula1>
-    </dataValidation>
-    <dataValidation sqref="C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - desconozco qué es el Fill Rate,Sí - sé qué es - pero no lo sigo,Sí - lo conozco y reviso ocasionalmente,Sí - lo reviso y gestiono activamente"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no lo conozco,Sí - lo conozco pero no lo monitoreo activamente,Sí - lo monitoreo activamente"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no conozco bien los requisitos de entrega,Conozco algunos pero tengo dudas frecuentes,Sí - los conozco y los cumplo correctamente"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - desconozco el proceso de agendamiento,Sí - pero tengo dudas frecuentes,Sí - lo sé y lo hago sin problemas"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no tengo esa información,Sí - pero solo cuando me avisan del quiebre,Sí - lo monitoreo regularmente"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No tengo visibilidad de mis quiebres,Sí - frecuentemente (más de 1 vez/mes),Sí - ocurren ocasionalmente,Sí - ocurren rara vez"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no tengo acceso,Sí - tengo acceso pero no sé para qué me sirve,Sí - lo uso para cosas básicas,Sí - lo uso y aprovecho sus reportes"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No lo hago,Una vez al mes,Semanalmente,Diariamente"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - nunca he escuchado ese nombre,Sí - lo conozco pero no lo uso,Sí - lo uso y sé cómo funciona"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no sé en qué tiendas estoy,Sé en cuáles tiendas estoy pero no lo actualizo,Sí - tengo información actualizada de mi presencia,Sí - además monitoreo el desempeño por local"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no conozco el proceso,He escuchado del proceso pero no lo conozco en detalle,Sí - lo conozco pero aún no he realizado alzas,Sí - he realizado alzas y conozco bien el proceso"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - nunca he participado,No - desconozco los requisitos,Sí - pero solo cuando me invitan,Sí - las busco activamente"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no entiendo la diferencia,Tengo una idea general pero no claridad total,Sí - los diferencio claramente"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"Soy yo quien administra la cuenta,Tengo KAM especializado para la cuenta,Tengo un conocido para la cuenta"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no lo conozco,Sí - he escuchado de él pero no sé cómo funciona,Sí - lo conozco y me interesa participar,Sí - ya participo o he participado en él"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no sé a quién acudir,Sí - tengo un contacto principal,Sí - tengo contactos según el tema"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - rara vez obtengo respuesta,Sí - a veces depende del tema,Sí - siempre obtengo respuesta oportuna"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no entiendo los motivos del rechazo,Sí - entiendo pero me cuesta corregirlo,Sí - entiendo y corrijo de inmediato"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no sé qué es,Sí - lo conozco pero no entiendo bien por qué,Sí - lo conozco y entiendo por qué se cobra"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"No - no sé qué es,Sí - lo conozco pero no entiendo bien por qué,Sí - lo conozco y entiendo por qué se cobra"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Respuesta no válida" error="Por favor, selecciona una de las opciones válidas sugeridas." promptTitle="Selecciona una opción" prompt="Haz clic en la flecha de la derecha y selecciona tu respuesta." type="list">
-      <formula1>"Sí - contamos con certificación,No - no tenemos certificación,En proceso de certificación"</formula1>
+    <dataValidation sqref="C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$A$1:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$B$1:$B$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="C13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$C$1:$C$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$D$1:$D$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="C15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$E$1:$E$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$F$1:$F$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$G$1:$G$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$H$1:$H$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$I$1:$I$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$J$1:$J$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="C21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$K$1:$K$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="C22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$L$1:$L$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$M$1:$M$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="C24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$N$1:$N$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="C25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$O$1:$O$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="C26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$P$1:$P$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$Q$1:$Q$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$R$1:$R$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="C29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$S$1:$S$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$T$1:$T$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$U$1:$U$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$V$1:$V$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$W$1:$W$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
+      <formula1>=Opciones_Encuesta!$X$1:$X$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:X6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Alimentos y Bebidas</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Menos de 6 meses</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Sí, ingresé y participé de las presentaciones y conversatorios.</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>No, desconozco qué es el Fill Rate</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>No, no lo conozco</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>No, no conozco bien los requisitos de entrega</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>No, desconozco el proceso de agendamiento</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>No, no tengo esa información</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>No tengo visibilidad de mis quiebres</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>No, no tengo acceso</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>No lo hago</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>No, nunca he escuchado ese nombre</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>No, no sé en qué tiendas estoy</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>No, no conozco el proceso</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>No, nunca he participado</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>No, no entiendo la diferencia</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Soy yo quien administra la cuenta</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>No, no lo conozco</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>No, no sé a quién acudir</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>No, rara vez obtengo respuesta</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>No, no entiendo los motivos del rechazo</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>No, no sé qué es</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>No, no sé qué es</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Sí, contamos con certificación</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Limpieza y Hogar</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Entre 6 meses y 1 año</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sí, pero no participé de nada adicional.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Sí, sé qué es, pero no lo sigo</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sí, lo conozco pero no lo monitoreo activamente</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Conozco algunos pero tengo dudas frecuentes</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Sí, pero tengo dudas frecuentes</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Sí, pero solo cuando me avisan del quiebre</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Sí, frecuentemente (más de 1 vez/mes)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Sí, tengo acceso pero no sé para qué me sirve</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Una vez al mes</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Sí, lo conozco pero no lo uso</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Sé en cuáles tiendas estoy pero no lo actualizo</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>He escuchado del proceso pero no lo conozco en detalle</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>No, desconozco los requisitos</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Tengo una idea general pero no claridad total</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Tengo KAM especializado para la cuenta</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Sí, he escuchado de él pero no sé cómo funciona</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Sí, tengo un contacto principal</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Sí, a veces depende del tema</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Sí, entiendo pero me cuesta corregirlo</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Sí, lo conozco pero no entiendo bien por qué</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Sí, lo conozco pero no entiendo bien por qué</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>No, no tenemos certificación</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cuidado Personal</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Entre 1 y 3 años</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No, entré por otra vía.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sí, lo conozco y reviso ocasionalmente</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sí, lo monitoreo activamente</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Sí, los conozco y los cumplo correctamente</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Sí, lo sé y lo hago sin problemas</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Sí, lo monitoreo regularmente</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Sí, ocurren ocasionalmente</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Sí, lo uso para cosas básicas</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Semanalmente</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Sí, lo uso y sé cómo funciona</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Sí, tengo información actualizada de mi presencia</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Sí, lo conozco pero aún no he realizado alzas</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Sí, pero solo cuando me invitan</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Sí, los diferencio claramente</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Tengo un conocido para la cuenta</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Sí, lo conozco y me interesa participar</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Sí, tengo contactos según el tema</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Sí, siempre obtengo respuesta oportuna</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Sí, entiendo y corrijo de inmediato</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Sí, lo conozco y entiendo por qué se cobra</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Sí, lo conozco y entiendo por qué se cobra</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>En proceso de certificación</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Textil y Ropa</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Más de 3 años</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sí, lo reviso y gestiono activamente</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Sí, ocurren rara vez</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Sí, lo uso y aprovecho sus reportes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Diariamente</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Sí, además monitoreo el desempeño por local</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Sí, he realizado alzas y conozco bien el proceso</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Sí, las busco activamente</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Sí, ya participo o he participado en él</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Electrónica</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Otra categoría</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Change excel to Walmart Navy design, restrict free text to 40 chars, lock sheet and keep yellow input cells editable
</commit_message>
<xml_diff>
--- a/ENCUESTA_MANUAL_PYME.xlsx
+++ b/ENCUESTA_MANUAL_PYME.xlsx
@@ -29,7 +29,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000C4A6E"/>
+      <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
@@ -81,8 +81,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0F2FE"/>
-        <bgColor rgb="00E0F2FE"/>
+        <fgColor rgb="00001E60"/>
+        <bgColor rgb="00001E60"/>
       </patternFill>
     </fill>
     <fill>
@@ -93,8 +93,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EC4899"/>
-        <bgColor rgb="00EC4899"/>
+        <fgColor rgb="00E0F2FE"/>
+        <bgColor rgb="00E0F2FE"/>
       </patternFill>
     </fill>
   </fills>
@@ -135,18 +135,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -598,7 +601,7 @@
       <c r="C10" s="8" t="n"/>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>[Escribe tu respuesta libremente]</t>
+          <t>[Escribe tu respuesta libremente - Máx 40 letras]</t>
         </is>
       </c>
     </row>
@@ -987,11 +990,15 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="E036"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D3"/>
   </mergeCells>
-  <dataValidations count="24">
+  <dataValidations count="25">
+    <dataValidation sqref="C5 C6 C7 C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Límite de caracteres (Máx 40)" error="La respuesta no puede quedar vacía ni exceder los 40 caracteres." promptTitle="Límite de caracteres" prompt="Por favor, ingresa tu respuesta de máximo 40 caracteres." type="textLength" operator="lessThanOrEqual">
+      <formula1>40</formula1>
+    </dataValidation>
     <dataValidation sqref="C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Selección inválida" error="Por favor, selecciona una de las opciones de la lista." promptTitle="Opciones de respuesta" prompt="Haz clic en la flecha de la derecha de la celda y selecciona tu respuesta." type="list">
       <formula1>=Opciones_Encuesta!$A$1:$A$6</formula1>
     </dataValidation>

</xml_diff>